<commit_message>
Bind Windows reference and final task specification
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R6a54b4941abb41ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="Rb88b89d1b9ed4be0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -410,7 +410,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R989b7ff817654853"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd56c372514a4667"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>